<commit_message>
Update: Updated testing script.
I added all the required updates to the testing script.  This made sure that the testing script was up to date as required.
</commit_message>
<xml_diff>
--- a/Timetracker Sheet.xlsx
+++ b/Timetracker Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11023"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexahope/Documents/GitHub/Ophelias-Oasis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D851B0-E2A5-A345-AA39-0818CCACC973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AD4F264-2070-AA41-A36A-F793F358C772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{DC8A763E-506D-49AB-8E26-20F95A084029}"/>
+    <workbookView xWindow="4680" yWindow="500" windowWidth="33720" windowHeight="19880" xr2:uid="{DC8A763E-506D-49AB-8E26-20F95A084029}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="49">
   <si>
     <t>Event:</t>
   </si>
@@ -180,6 +180,12 @@
   </si>
   <si>
     <t xml:space="preserve">During this time I added some of the testing script information back.  This made sure the program worked as intended.  The program would work properly if I did that. However, it did not appear to be full done which was the source of my worry.  </t>
+  </si>
+  <si>
+    <t>3:40 PM - 5:00 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">During this time I added some entries into the testing script.  This made sure the testing script was up to date with all the required entries.  </t>
   </si>
 </sst>
 </file>
@@ -1026,7 +1032,24 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C25" s="4"/>
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="4">
+        <v>80</v>
+      </c>
+      <c r="D25" s="2">
+        <v>46322</v>
+      </c>
+      <c r="E25" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C26" s="4"/>

</xml_diff>